<commit_message>
docs: update README & test tracker
</commit_message>
<xml_diff>
--- a/docs/SylvanShield_TestCases.xlsx
+++ b/docs/SylvanShield_TestCases.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/luuuuuuke/Desktop/SylvanShield/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C074A5F2-C84E-DD49-9F6E-200BE0F9C0D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55C80BF0-C472-9849-9E80-1EA8A05B724E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11040" yWindow="2080" windowWidth="30240" windowHeight="17840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2140" yWindow="1780" windowWidth="30240" windowHeight="17840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Test Execution" sheetId="1" r:id="rId1"/>
@@ -262,10 +262,6 @@
     <t>Status = GRACE_PERIOD. GRACE_PERIOD_MS = 5000ms.</t>
   </si>
   <si>
-    <t>1. Enter grace period
-2. Wait 5 seconds without action</t>
-  </si>
-  <si>
     <t>Status = ALERT_SENT. Card turns red. Emergency email received in inbox</t>
   </si>
   <si>
@@ -902,6 +898,10 @@
   </si>
   <si>
     <t>✅Pass</t>
+  </si>
+  <si>
+    <t>1. Enter grace period
+2. Wait 5 seconds without action(for testing)</t>
   </si>
 </sst>
 </file>
@@ -1567,10 +1567,10 @@
       </c>
       <c r="H3" s="7"/>
       <c r="I3" s="8" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="J3" s="28" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="K3" s="27"/>
       <c r="L3" s="27"/>
@@ -1605,7 +1605,7 @@
       </c>
       <c r="H4" s="7"/>
       <c r="I4" s="8" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="5" spans="1:18" ht="52" customHeight="1" x14ac:dyDescent="0.2">
@@ -1632,7 +1632,7 @@
       </c>
       <c r="H5" s="7"/>
       <c r="I5" s="8" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="6" spans="1:18" ht="52" customHeight="1" x14ac:dyDescent="0.2">
@@ -1895,10 +1895,10 @@
         <v>74</v>
       </c>
       <c r="F15" s="6" t="s">
+        <v>276</v>
+      </c>
+      <c r="G15" s="6" t="s">
         <v>75</v>
-      </c>
-      <c r="G15" s="6" t="s">
-        <v>76</v>
       </c>
       <c r="H15" s="7"/>
       <c r="I15" s="8" t="s">
@@ -1907,25 +1907,25 @@
     </row>
     <row r="16" spans="1:18" ht="52" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B16" s="3" t="s">
         <v>43</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D16" s="5" t="s">
         <v>13</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F16" s="6" t="s">
         <v>70</v>
       </c>
       <c r="G16" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H16" s="7"/>
       <c r="I16" s="8" t="s">
@@ -1934,25 +1934,25 @@
     </row>
     <row r="17" spans="1:9" ht="52" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B17" s="3" t="s">
         <v>43</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D17" s="5" t="s">
         <v>13</v>
       </c>
       <c r="E17" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="F17" s="6" t="s">
         <v>83</v>
       </c>
-      <c r="F17" s="6" t="s">
+      <c r="G17" s="6" t="s">
         <v>84</v>
-      </c>
-      <c r="G17" s="6" t="s">
-        <v>85</v>
       </c>
       <c r="H17" s="7"/>
       <c r="I17" s="8" t="s">
@@ -1961,25 +1961,25 @@
     </row>
     <row r="18" spans="1:9" ht="52" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="9" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B18" s="10" t="s">
         <v>43</v>
       </c>
       <c r="C18" s="11" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D18" s="12" t="s">
         <v>29</v>
       </c>
       <c r="E18" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="F18" s="6" t="s">
         <v>88</v>
       </c>
-      <c r="F18" s="6" t="s">
+      <c r="G18" s="6" t="s">
         <v>89</v>
-      </c>
-      <c r="G18" s="6" t="s">
-        <v>90</v>
       </c>
       <c r="H18" s="7"/>
       <c r="I18" s="8" t="s">
@@ -1988,25 +1988,25 @@
     </row>
     <row r="19" spans="1:9" ht="52" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="B19" s="3" t="s">
         <v>91</v>
       </c>
-      <c r="B19" s="3" t="s">
+      <c r="C19" s="4" t="s">
         <v>92</v>
-      </c>
-      <c r="C19" s="4" t="s">
-        <v>93</v>
       </c>
       <c r="D19" s="5" t="s">
         <v>13</v>
       </c>
       <c r="E19" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="F19" s="6" t="s">
         <v>94</v>
       </c>
-      <c r="F19" s="6" t="s">
+      <c r="G19" s="6" t="s">
         <v>95</v>
-      </c>
-      <c r="G19" s="6" t="s">
-        <v>96</v>
       </c>
       <c r="H19" s="7"/>
       <c r="I19" s="8" t="s">
@@ -2015,25 +2015,25 @@
     </row>
     <row r="20" spans="1:9" ht="52" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="B20" s="10" t="s">
+        <v>91</v>
+      </c>
+      <c r="C20" s="11" t="s">
         <v>97</v>
-      </c>
-      <c r="B20" s="10" t="s">
-        <v>92</v>
-      </c>
-      <c r="C20" s="11" t="s">
-        <v>98</v>
       </c>
       <c r="D20" s="12" t="s">
         <v>29</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="F20" s="6" t="s">
         <v>56</v>
       </c>
       <c r="G20" s="6" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H20" s="7"/>
       <c r="I20" s="8" t="s">
@@ -2042,25 +2042,25 @@
     </row>
     <row r="21" spans="1:9" ht="52" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="C21" s="4" t="s">
         <v>101</v>
-      </c>
-      <c r="B21" s="3" t="s">
-        <v>92</v>
-      </c>
-      <c r="C21" s="4" t="s">
-        <v>102</v>
       </c>
       <c r="D21" s="5" t="s">
         <v>13</v>
       </c>
       <c r="E21" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="F21" s="6" t="s">
         <v>103</v>
       </c>
-      <c r="F21" s="6" t="s">
+      <c r="G21" s="6" t="s">
         <v>104</v>
-      </c>
-      <c r="G21" s="6" t="s">
-        <v>105</v>
       </c>
       <c r="H21" s="7"/>
       <c r="I21" s="8" t="s">
@@ -2069,25 +2069,25 @@
     </row>
     <row r="22" spans="1:9" ht="52" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="C22" s="4" t="s">
         <v>106</v>
-      </c>
-      <c r="B22" s="3" t="s">
-        <v>92</v>
-      </c>
-      <c r="C22" s="4" t="s">
-        <v>107</v>
       </c>
       <c r="D22" s="5" t="s">
         <v>13</v>
       </c>
       <c r="E22" s="6" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F22" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="G22" s="6" t="s">
         <v>108</v>
-      </c>
-      <c r="G22" s="6" t="s">
-        <v>109</v>
       </c>
       <c r="H22" s="7"/>
       <c r="I22" s="8" t="s">
@@ -2096,25 +2096,25 @@
     </row>
     <row r="23" spans="1:9" ht="52" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="9" t="s">
+        <v>109</v>
+      </c>
+      <c r="B23" s="10" t="s">
+        <v>91</v>
+      </c>
+      <c r="C23" s="11" t="s">
         <v>110</v>
-      </c>
-      <c r="B23" s="10" t="s">
-        <v>92</v>
-      </c>
-      <c r="C23" s="11" t="s">
-        <v>111</v>
       </c>
       <c r="D23" s="12" t="s">
         <v>29</v>
       </c>
       <c r="E23" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="F23" s="6" t="s">
         <v>112</v>
       </c>
-      <c r="F23" s="6" t="s">
+      <c r="G23" s="6" t="s">
         <v>113</v>
-      </c>
-      <c r="G23" s="6" t="s">
-        <v>114</v>
       </c>
       <c r="H23" s="7"/>
       <c r="I23" s="8" t="s">
@@ -2123,25 +2123,25 @@
     </row>
     <row r="24" spans="1:9" ht="52" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="9" t="s">
+        <v>114</v>
+      </c>
+      <c r="B24" s="10" t="s">
+        <v>91</v>
+      </c>
+      <c r="C24" s="11" t="s">
         <v>115</v>
-      </c>
-      <c r="B24" s="10" t="s">
-        <v>92</v>
-      </c>
-      <c r="C24" s="11" t="s">
-        <v>116</v>
       </c>
       <c r="D24" s="12" t="s">
         <v>29</v>
       </c>
       <c r="E24" s="6" t="s">
+        <v>116</v>
+      </c>
+      <c r="F24" s="6" t="s">
         <v>117</v>
       </c>
-      <c r="F24" s="6" t="s">
+      <c r="G24" s="6" t="s">
         <v>118</v>
-      </c>
-      <c r="G24" s="6" t="s">
-        <v>119</v>
       </c>
       <c r="H24" s="7"/>
       <c r="I24" s="8" t="s">
@@ -2150,25 +2150,25 @@
     </row>
     <row r="25" spans="1:9" ht="52" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="B25" s="3" t="s">
         <v>120</v>
       </c>
-      <c r="B25" s="3" t="s">
+      <c r="C25" s="4" t="s">
         <v>121</v>
-      </c>
-      <c r="C25" s="4" t="s">
-        <v>122</v>
       </c>
       <c r="D25" s="5" t="s">
         <v>13</v>
       </c>
       <c r="E25" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="F25" s="6" t="s">
         <v>123</v>
       </c>
-      <c r="F25" s="6" t="s">
+      <c r="G25" s="6" t="s">
         <v>124</v>
-      </c>
-      <c r="G25" s="6" t="s">
-        <v>125</v>
       </c>
       <c r="H25" s="7"/>
       <c r="I25" s="8" t="s">
@@ -2177,25 +2177,25 @@
     </row>
     <row r="26" spans="1:9" ht="52" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="B26" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="C26" s="4" t="s">
         <v>126</v>
-      </c>
-      <c r="B26" s="3" t="s">
-        <v>121</v>
-      </c>
-      <c r="C26" s="4" t="s">
-        <v>127</v>
       </c>
       <c r="D26" s="5" t="s">
         <v>13</v>
       </c>
       <c r="E26" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="F26" s="6" t="s">
         <v>128</v>
       </c>
-      <c r="F26" s="6" t="s">
+      <c r="G26" s="6" t="s">
         <v>129</v>
-      </c>
-      <c r="G26" s="6" t="s">
-        <v>130</v>
       </c>
       <c r="H26" s="7"/>
       <c r="I26" s="8" t="s">
@@ -2204,25 +2204,25 @@
     </row>
     <row r="27" spans="1:9" ht="52" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="B27" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="C27" s="4" t="s">
         <v>131</v>
-      </c>
-      <c r="B27" s="3" t="s">
-        <v>121</v>
-      </c>
-      <c r="C27" s="4" t="s">
-        <v>132</v>
       </c>
       <c r="D27" s="5" t="s">
         <v>13</v>
       </c>
       <c r="E27" s="6" t="s">
+        <v>132</v>
+      </c>
+      <c r="F27" s="6" t="s">
         <v>133</v>
       </c>
-      <c r="F27" s="6" t="s">
+      <c r="G27" s="6" t="s">
         <v>134</v>
-      </c>
-      <c r="G27" s="6" t="s">
-        <v>135</v>
       </c>
       <c r="H27" s="7"/>
       <c r="I27" s="8" t="s">
@@ -2231,79 +2231,79 @@
     </row>
     <row r="28" spans="1:9" ht="52" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="9" t="s">
+        <v>135</v>
+      </c>
+      <c r="B28" s="10" t="s">
+        <v>120</v>
+      </c>
+      <c r="C28" s="11" t="s">
         <v>136</v>
-      </c>
-      <c r="B28" s="10" t="s">
-        <v>121</v>
-      </c>
-      <c r="C28" s="11" t="s">
-        <v>137</v>
       </c>
       <c r="D28" s="12" t="s">
         <v>29</v>
       </c>
       <c r="E28" s="6" t="s">
+        <v>137</v>
+      </c>
+      <c r="F28" s="6" t="s">
         <v>138</v>
       </c>
-      <c r="F28" s="6" t="s">
+      <c r="G28" s="6" t="s">
         <v>139</v>
-      </c>
-      <c r="G28" s="6" t="s">
-        <v>140</v>
       </c>
       <c r="H28" s="7"/>
       <c r="I28" s="8" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="29" spans="1:9" ht="52" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="13" t="s">
+        <v>140</v>
+      </c>
+      <c r="B29" s="14" t="s">
+        <v>120</v>
+      </c>
+      <c r="C29" s="15" t="s">
         <v>141</v>
       </c>
-      <c r="B29" s="14" t="s">
-        <v>121</v>
-      </c>
-      <c r="C29" s="15" t="s">
+      <c r="D29" s="16" t="s">
         <v>142</v>
       </c>
-      <c r="D29" s="16" t="s">
+      <c r="E29" s="6" t="s">
         <v>143</v>
       </c>
-      <c r="E29" s="6" t="s">
+      <c r="F29" s="6" t="s">
         <v>144</v>
       </c>
-      <c r="F29" s="6" t="s">
+      <c r="G29" s="6" t="s">
         <v>145</v>
-      </c>
-      <c r="G29" s="6" t="s">
-        <v>146</v>
       </c>
       <c r="H29" s="7"/>
       <c r="I29" s="8" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="30" spans="1:9" ht="52" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="B30" s="3" t="s">
         <v>147</v>
       </c>
-      <c r="B30" s="3" t="s">
+      <c r="C30" s="4" t="s">
         <v>148</v>
-      </c>
-      <c r="C30" s="4" t="s">
-        <v>149</v>
       </c>
       <c r="D30" s="5" t="s">
         <v>13</v>
       </c>
       <c r="E30" s="6" t="s">
+        <v>149</v>
+      </c>
+      <c r="F30" s="6" t="s">
         <v>150</v>
       </c>
-      <c r="F30" s="6" t="s">
+      <c r="G30" s="6" t="s">
         <v>151</v>
-      </c>
-      <c r="G30" s="6" t="s">
-        <v>152</v>
       </c>
       <c r="H30" s="7"/>
       <c r="I30" s="8" t="s">
@@ -2312,25 +2312,25 @@
     </row>
     <row r="31" spans="1:9" ht="52" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="B31" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="C31" s="4" t="s">
         <v>153</v>
-      </c>
-      <c r="B31" s="3" t="s">
-        <v>148</v>
-      </c>
-      <c r="C31" s="4" t="s">
-        <v>154</v>
       </c>
       <c r="D31" s="5" t="s">
         <v>13</v>
       </c>
       <c r="E31" s="6" t="s">
+        <v>154</v>
+      </c>
+      <c r="F31" s="6" t="s">
         <v>155</v>
       </c>
-      <c r="F31" s="6" t="s">
+      <c r="G31" s="6" t="s">
         <v>156</v>
-      </c>
-      <c r="G31" s="6" t="s">
-        <v>157</v>
       </c>
       <c r="H31" s="7"/>
       <c r="I31" s="8" t="s">
@@ -2339,25 +2339,25 @@
     </row>
     <row r="32" spans="1:9" ht="52" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="B32" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="C32" s="4" t="s">
         <v>158</v>
-      </c>
-      <c r="B32" s="3" t="s">
-        <v>148</v>
-      </c>
-      <c r="C32" s="4" t="s">
-        <v>159</v>
       </c>
       <c r="D32" s="5" t="s">
         <v>13</v>
       </c>
       <c r="E32" s="6" t="s">
+        <v>159</v>
+      </c>
+      <c r="F32" s="6" t="s">
         <v>160</v>
       </c>
-      <c r="F32" s="6" t="s">
+      <c r="G32" s="6" t="s">
         <v>161</v>
-      </c>
-      <c r="G32" s="6" t="s">
-        <v>162</v>
       </c>
       <c r="H32" s="7"/>
       <c r="I32" s="8" t="s">
@@ -2366,25 +2366,25 @@
     </row>
     <row r="33" spans="1:9" ht="52" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="9" t="s">
+        <v>162</v>
+      </c>
+      <c r="B33" s="10" t="s">
+        <v>147</v>
+      </c>
+      <c r="C33" s="11" t="s">
         <v>163</v>
-      </c>
-      <c r="B33" s="10" t="s">
-        <v>148</v>
-      </c>
-      <c r="C33" s="11" t="s">
-        <v>164</v>
       </c>
       <c r="D33" s="12" t="s">
         <v>29</v>
       </c>
       <c r="E33" s="6" t="s">
+        <v>164</v>
+      </c>
+      <c r="F33" s="6" t="s">
         <v>165</v>
       </c>
-      <c r="F33" s="6" t="s">
+      <c r="G33" s="6" t="s">
         <v>166</v>
-      </c>
-      <c r="G33" s="6" t="s">
-        <v>167</v>
       </c>
       <c r="H33" s="7"/>
       <c r="I33" s="8" t="s">
@@ -2393,25 +2393,25 @@
     </row>
     <row r="34" spans="1:9" ht="52" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="9" t="s">
+        <v>167</v>
+      </c>
+      <c r="B34" s="10" t="s">
+        <v>147</v>
+      </c>
+      <c r="C34" s="11" t="s">
         <v>168</v>
-      </c>
-      <c r="B34" s="10" t="s">
-        <v>148</v>
-      </c>
-      <c r="C34" s="11" t="s">
-        <v>169</v>
       </c>
       <c r="D34" s="12" t="s">
         <v>29</v>
       </c>
       <c r="E34" s="6" t="s">
+        <v>169</v>
+      </c>
+      <c r="F34" s="6" t="s">
         <v>170</v>
       </c>
-      <c r="F34" s="6" t="s">
+      <c r="G34" s="6" t="s">
         <v>171</v>
-      </c>
-      <c r="G34" s="6" t="s">
-        <v>172</v>
       </c>
       <c r="H34" s="7"/>
       <c r="I34" s="8" t="s">
@@ -2420,25 +2420,25 @@
     </row>
     <row r="35" spans="1:9" ht="52" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="13" t="s">
+        <v>172</v>
+      </c>
+      <c r="B35" s="14" t="s">
+        <v>147</v>
+      </c>
+      <c r="C35" s="15" t="s">
         <v>173</v>
       </c>
-      <c r="B35" s="14" t="s">
-        <v>148</v>
-      </c>
-      <c r="C35" s="15" t="s">
+      <c r="D35" s="16" t="s">
+        <v>142</v>
+      </c>
+      <c r="E35" s="6" t="s">
         <v>174</v>
       </c>
-      <c r="D35" s="16" t="s">
-        <v>143</v>
-      </c>
-      <c r="E35" s="6" t="s">
+      <c r="F35" s="6" t="s">
         <v>175</v>
       </c>
-      <c r="F35" s="6" t="s">
+      <c r="G35" s="6" t="s">
         <v>176</v>
-      </c>
-      <c r="G35" s="6" t="s">
-        <v>177</v>
       </c>
       <c r="H35" s="7"/>
       <c r="I35" s="8" t="s">
@@ -2447,25 +2447,25 @@
     </row>
     <row r="36" spans="1:9" ht="52" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="B36" s="3" t="s">
         <v>178</v>
       </c>
-      <c r="B36" s="3" t="s">
+      <c r="C36" s="4" t="s">
         <v>179</v>
-      </c>
-      <c r="C36" s="4" t="s">
-        <v>180</v>
       </c>
       <c r="D36" s="5" t="s">
         <v>13</v>
       </c>
       <c r="E36" s="6" t="s">
+        <v>180</v>
+      </c>
+      <c r="F36" s="6" t="s">
         <v>181</v>
       </c>
-      <c r="F36" s="6" t="s">
+      <c r="G36" s="6" t="s">
         <v>182</v>
-      </c>
-      <c r="G36" s="6" t="s">
-        <v>183</v>
       </c>
       <c r="H36" s="7"/>
       <c r="I36" s="8" t="s">
@@ -2474,25 +2474,25 @@
     </row>
     <row r="37" spans="1:9" ht="52" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="2" t="s">
+        <v>183</v>
+      </c>
+      <c r="B37" s="3" t="s">
+        <v>178</v>
+      </c>
+      <c r="C37" s="4" t="s">
         <v>184</v>
-      </c>
-      <c r="B37" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="C37" s="4" t="s">
-        <v>185</v>
       </c>
       <c r="D37" s="5" t="s">
         <v>13</v>
       </c>
       <c r="E37" s="6" t="s">
+        <v>185</v>
+      </c>
+      <c r="F37" s="6" t="s">
         <v>186</v>
       </c>
-      <c r="F37" s="6" t="s">
+      <c r="G37" s="6" t="s">
         <v>187</v>
-      </c>
-      <c r="G37" s="6" t="s">
-        <v>188</v>
       </c>
       <c r="H37" s="7"/>
       <c r="I37" s="8" t="s">
@@ -2501,25 +2501,25 @@
     </row>
     <row r="38" spans="1:9" ht="52" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="9" t="s">
+        <v>188</v>
+      </c>
+      <c r="B38" s="10" t="s">
+        <v>178</v>
+      </c>
+      <c r="C38" s="11" t="s">
         <v>189</v>
-      </c>
-      <c r="B38" s="10" t="s">
-        <v>179</v>
-      </c>
-      <c r="C38" s="11" t="s">
-        <v>190</v>
       </c>
       <c r="D38" s="12" t="s">
         <v>29</v>
       </c>
       <c r="E38" s="6" t="s">
+        <v>190</v>
+      </c>
+      <c r="F38" s="6" t="s">
         <v>191</v>
       </c>
-      <c r="F38" s="6" t="s">
+      <c r="G38" s="6" t="s">
         <v>192</v>
-      </c>
-      <c r="G38" s="6" t="s">
-        <v>193</v>
       </c>
       <c r="H38" s="7"/>
       <c r="I38" s="8" t="s">
@@ -2528,25 +2528,25 @@
     </row>
     <row r="39" spans="1:9" ht="52" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="9" t="s">
+        <v>193</v>
+      </c>
+      <c r="B39" s="10" t="s">
+        <v>178</v>
+      </c>
+      <c r="C39" s="11" t="s">
         <v>194</v>
-      </c>
-      <c r="B39" s="10" t="s">
-        <v>179</v>
-      </c>
-      <c r="C39" s="11" t="s">
-        <v>195</v>
       </c>
       <c r="D39" s="12" t="s">
         <v>29</v>
       </c>
       <c r="E39" s="6" t="s">
+        <v>195</v>
+      </c>
+      <c r="F39" s="6" t="s">
         <v>196</v>
       </c>
-      <c r="F39" s="6" t="s">
+      <c r="G39" s="6" t="s">
         <v>197</v>
-      </c>
-      <c r="G39" s="6" t="s">
-        <v>198</v>
       </c>
       <c r="H39" s="7"/>
       <c r="I39" s="8" t="s">
@@ -2555,25 +2555,25 @@
     </row>
     <row r="40" spans="1:9" ht="52" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="13" t="s">
+        <v>198</v>
+      </c>
+      <c r="B40" s="14" t="s">
+        <v>178</v>
+      </c>
+      <c r="C40" s="15" t="s">
         <v>199</v>
       </c>
-      <c r="B40" s="14" t="s">
-        <v>179</v>
-      </c>
-      <c r="C40" s="15" t="s">
+      <c r="D40" s="16" t="s">
+        <v>142</v>
+      </c>
+      <c r="E40" s="6" t="s">
         <v>200</v>
       </c>
-      <c r="D40" s="16" t="s">
-        <v>143</v>
-      </c>
-      <c r="E40" s="6" t="s">
+      <c r="F40" s="6" t="s">
         <v>201</v>
       </c>
-      <c r="F40" s="6" t="s">
+      <c r="G40" s="6" t="s">
         <v>202</v>
-      </c>
-      <c r="G40" s="6" t="s">
-        <v>203</v>
       </c>
       <c r="H40" s="7"/>
       <c r="I40" s="8" t="s">
@@ -2582,25 +2582,25 @@
     </row>
     <row r="41" spans="1:9" ht="52" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="B41" s="3" t="s">
         <v>204</v>
       </c>
-      <c r="B41" s="3" t="s">
+      <c r="C41" s="4" t="s">
         <v>205</v>
-      </c>
-      <c r="C41" s="4" t="s">
-        <v>206</v>
       </c>
       <c r="D41" s="5" t="s">
         <v>13</v>
       </c>
       <c r="E41" s="6" t="s">
+        <v>206</v>
+      </c>
+      <c r="F41" s="6" t="s">
         <v>207</v>
       </c>
-      <c r="F41" s="6" t="s">
+      <c r="G41" s="6" t="s">
         <v>208</v>
-      </c>
-      <c r="G41" s="6" t="s">
-        <v>209</v>
       </c>
       <c r="H41" s="7"/>
       <c r="I41" s="8" t="s">
@@ -2609,25 +2609,25 @@
     </row>
     <row r="42" spans="1:9" ht="52" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="B42" s="3" t="s">
+        <v>204</v>
+      </c>
+      <c r="C42" s="4" t="s">
         <v>210</v>
-      </c>
-      <c r="B42" s="3" t="s">
-        <v>205</v>
-      </c>
-      <c r="C42" s="4" t="s">
-        <v>211</v>
       </c>
       <c r="D42" s="5" t="s">
         <v>13</v>
       </c>
       <c r="E42" s="6" t="s">
+        <v>211</v>
+      </c>
+      <c r="F42" s="6" t="s">
         <v>212</v>
       </c>
-      <c r="F42" s="6" t="s">
+      <c r="G42" s="6" t="s">
         <v>213</v>
-      </c>
-      <c r="G42" s="6" t="s">
-        <v>214</v>
       </c>
       <c r="H42" s="7"/>
       <c r="I42" s="8" t="s">
@@ -2636,25 +2636,25 @@
     </row>
     <row r="43" spans="1:9" ht="52" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="9" t="s">
+        <v>214</v>
+      </c>
+      <c r="B43" s="10" t="s">
+        <v>204</v>
+      </c>
+      <c r="C43" s="11" t="s">
         <v>215</v>
-      </c>
-      <c r="B43" s="10" t="s">
-        <v>205</v>
-      </c>
-      <c r="C43" s="11" t="s">
-        <v>216</v>
       </c>
       <c r="D43" s="12" t="s">
         <v>29</v>
       </c>
       <c r="E43" s="6" t="s">
+        <v>216</v>
+      </c>
+      <c r="F43" s="6" t="s">
         <v>217</v>
       </c>
-      <c r="F43" s="6" t="s">
+      <c r="G43" s="6" t="s">
         <v>218</v>
-      </c>
-      <c r="G43" s="6" t="s">
-        <v>219</v>
       </c>
       <c r="H43" s="7"/>
       <c r="I43" s="8" t="s">
@@ -2663,25 +2663,25 @@
     </row>
     <row r="44" spans="1:9" ht="52" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="13" t="s">
+        <v>219</v>
+      </c>
+      <c r="B44" s="14" t="s">
+        <v>204</v>
+      </c>
+      <c r="C44" s="15" t="s">
         <v>220</v>
       </c>
-      <c r="B44" s="14" t="s">
-        <v>205</v>
-      </c>
-      <c r="C44" s="15" t="s">
+      <c r="D44" s="16" t="s">
+        <v>142</v>
+      </c>
+      <c r="E44" s="6" t="s">
         <v>221</v>
       </c>
-      <c r="D44" s="16" t="s">
-        <v>143</v>
-      </c>
-      <c r="E44" s="6" t="s">
+      <c r="F44" s="6" t="s">
         <v>222</v>
       </c>
-      <c r="F44" s="6" t="s">
+      <c r="G44" s="6" t="s">
         <v>223</v>
-      </c>
-      <c r="G44" s="6" t="s">
-        <v>224</v>
       </c>
       <c r="H44" s="7"/>
       <c r="I44" s="8" t="s">
@@ -2690,25 +2690,25 @@
     </row>
     <row r="45" spans="1:9" ht="52" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="2" t="s">
+        <v>224</v>
+      </c>
+      <c r="B45" s="3" t="s">
         <v>225</v>
       </c>
-      <c r="B45" s="3" t="s">
+      <c r="C45" s="4" t="s">
         <v>226</v>
-      </c>
-      <c r="C45" s="4" t="s">
-        <v>227</v>
       </c>
       <c r="D45" s="5" t="s">
         <v>13</v>
       </c>
       <c r="E45" s="6" t="s">
+        <v>227</v>
+      </c>
+      <c r="F45" s="6" t="s">
         <v>228</v>
       </c>
-      <c r="F45" s="6" t="s">
+      <c r="G45" s="6" t="s">
         <v>229</v>
-      </c>
-      <c r="G45" s="6" t="s">
-        <v>230</v>
       </c>
       <c r="H45" s="7"/>
       <c r="I45" s="8" t="s">
@@ -2717,25 +2717,25 @@
     </row>
     <row r="46" spans="1:9" ht="52" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="B46" s="3" t="s">
+        <v>225</v>
+      </c>
+      <c r="C46" s="4" t="s">
         <v>231</v>
-      </c>
-      <c r="B46" s="3" t="s">
-        <v>226</v>
-      </c>
-      <c r="C46" s="4" t="s">
-        <v>232</v>
       </c>
       <c r="D46" s="5" t="s">
         <v>13</v>
       </c>
       <c r="E46" s="6" t="s">
+        <v>232</v>
+      </c>
+      <c r="F46" s="6" t="s">
         <v>233</v>
       </c>
-      <c r="F46" s="6" t="s">
+      <c r="G46" s="6" t="s">
         <v>234</v>
-      </c>
-      <c r="G46" s="6" t="s">
-        <v>235</v>
       </c>
       <c r="H46" s="7"/>
       <c r="I46" s="8" t="s">
@@ -2744,25 +2744,25 @@
     </row>
     <row r="47" spans="1:9" ht="52" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="9" t="s">
+        <v>235</v>
+      </c>
+      <c r="B47" s="10" t="s">
+        <v>225</v>
+      </c>
+      <c r="C47" s="11" t="s">
         <v>236</v>
-      </c>
-      <c r="B47" s="10" t="s">
-        <v>226</v>
-      </c>
-      <c r="C47" s="11" t="s">
-        <v>237</v>
       </c>
       <c r="D47" s="12" t="s">
         <v>29</v>
       </c>
       <c r="E47" s="6" t="s">
+        <v>237</v>
+      </c>
+      <c r="F47" s="6" t="s">
         <v>238</v>
       </c>
-      <c r="F47" s="6" t="s">
+      <c r="G47" s="6" t="s">
         <v>239</v>
-      </c>
-      <c r="G47" s="6" t="s">
-        <v>240</v>
       </c>
       <c r="H47" s="7"/>
       <c r="I47" s="8" t="s">
@@ -2771,25 +2771,25 @@
     </row>
     <row r="48" spans="1:9" ht="52" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="13" t="s">
+        <v>240</v>
+      </c>
+      <c r="B48" s="14" t="s">
+        <v>225</v>
+      </c>
+      <c r="C48" s="15" t="s">
         <v>241</v>
       </c>
-      <c r="B48" s="14" t="s">
-        <v>226</v>
-      </c>
-      <c r="C48" s="15" t="s">
+      <c r="D48" s="16" t="s">
+        <v>142</v>
+      </c>
+      <c r="E48" s="6" t="s">
+        <v>237</v>
+      </c>
+      <c r="F48" s="6" t="s">
         <v>242</v>
       </c>
-      <c r="D48" s="16" t="s">
-        <v>143</v>
-      </c>
-      <c r="E48" s="6" t="s">
-        <v>238</v>
-      </c>
-      <c r="F48" s="6" t="s">
+      <c r="G48" s="6" t="s">
         <v>243</v>
-      </c>
-      <c r="G48" s="6" t="s">
-        <v>244</v>
       </c>
       <c r="H48" s="7"/>
       <c r="I48" s="8" t="s">
@@ -2815,9 +2815,12 @@
       <formula>NOT(ISERROR(SEARCH("Partial",I3)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="working， aiefnf, " sqref="I3:I48" xr:uid="{04D47839-6082-1048-8208-F2A0A2181C3F}">
+  <dataValidations count="2">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="working， aiefnf, " sqref="I3 I5:I48" xr:uid="{04D47839-6082-1048-8208-F2A0A2181C3F}">
       <formula1>"✅Pass, ❌Fail, ⚠️Part, 🔲Not Tested"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="working， aiefnf, " sqref="I4" xr:uid="{774F449D-BE54-8E44-81C1-4F69A73EFBEC}">
+      <formula1>"✅Pass, ❌Fail, ⚠️Partial, 🔲Not Tested"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2836,7 +2839,7 @@
   <sheetData>
     <row r="1" spans="1:6" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="26" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B1" s="27"/>
       <c r="C1" s="27"/>
@@ -2846,7 +2849,7 @@
     </row>
     <row r="2" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="29" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="B2" s="27"/>
       <c r="C2" s="27"/>
@@ -2859,19 +2862,19 @@
         <v>2</v>
       </c>
       <c r="B4" s="1" t="s">
+        <v>247</v>
+      </c>
+      <c r="C4" s="1" t="s">
         <v>248</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="D4" s="1" t="s">
         <v>249</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="E4" s="1" t="s">
         <v>250</v>
       </c>
-      <c r="E4" s="1" t="s">
+      <c r="F4" s="1" t="s">
         <v>251</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>252</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -2882,16 +2885,16 @@
         <v>6</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -2902,161 +2905,161 @@
         <v>10</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="17" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B7" s="18">
         <v>6</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="F7" s="8" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="17" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B8" s="18">
         <v>5</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="F8" s="8" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="17" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B9" s="18">
         <v>6</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="F9" s="8" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="17" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="B10" s="18">
         <v>5</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="F10" s="8" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="17" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="B11" s="18">
         <v>4</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="F11" s="8" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="17" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B12" s="18">
         <v>4</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="D12" s="8" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="E12" s="8" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="F12" s="8" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="19" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="B13" s="20">
         <v>46</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="D13" s="8" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="F13" s="8" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="30" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="B15" s="27"/>
       <c r="C15" s="27"/>
@@ -3066,7 +3069,7 @@
     </row>
     <row r="16" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="2" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="B16" s="21">
         <v>28</v>
@@ -3078,7 +3081,7 @@
     </row>
     <row r="17" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="9" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="B17" s="22">
         <v>13</v>
@@ -3090,7 +3093,7 @@
     </row>
     <row r="18" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="13" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="B18" s="23">
         <v>5</v>
@@ -3123,7 +3126,7 @@
   <sheetData>
     <row r="1" spans="1:4" ht="26" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="31" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="B1" s="27"/>
       <c r="C1" s="27"/>
@@ -3131,16 +3134,16 @@
     </row>
     <row r="2" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
+        <v>259</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>260</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>261</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>9</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="22" customHeight="1" x14ac:dyDescent="0.2">
@@ -3148,7 +3151,7 @@
         <v>1</v>
       </c>
       <c r="B3" s="25" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="C3" s="8" t="s">
         <v>17</v>
@@ -3160,7 +3163,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="25" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="C4" s="8" t="s">
         <v>17</v>
@@ -3172,7 +3175,7 @@
         <v>3</v>
       </c>
       <c r="B5" s="25" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="C5" s="8" t="s">
         <v>17</v>
@@ -3184,7 +3187,7 @@
         <v>4</v>
       </c>
       <c r="B6" s="25" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="C6" s="8" t="s">
         <v>17</v>
@@ -3196,7 +3199,7 @@
         <v>5</v>
       </c>
       <c r="B7" s="25" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="C7" s="8" t="s">
         <v>17</v>
@@ -3208,7 +3211,7 @@
         <v>6</v>
       </c>
       <c r="B8" s="25" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="C8" s="8" t="s">
         <v>17</v>
@@ -3220,7 +3223,7 @@
         <v>7</v>
       </c>
       <c r="B9" s="25" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="C9" s="8" t="s">
         <v>17</v>
@@ -3232,7 +3235,7 @@
         <v>8</v>
       </c>
       <c r="B10" s="25" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="C10" s="8" t="s">
         <v>17</v>
@@ -3244,7 +3247,7 @@
         <v>9</v>
       </c>
       <c r="B11" s="25" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="C11" s="8" t="s">
         <v>17</v>
@@ -3256,7 +3259,7 @@
         <v>10</v>
       </c>
       <c r="B12" s="25" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="C12" s="8" t="s">
         <v>17</v>
@@ -3268,7 +3271,7 @@
         <v>11</v>
       </c>
       <c r="B13" s="25" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="C13" s="8" t="s">
         <v>17</v>
@@ -3280,7 +3283,7 @@
         <v>12</v>
       </c>
       <c r="B14" s="25" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="C14" s="8" t="s">
         <v>17</v>

</xml_diff>